<commit_message>
Phase 11F Batch 3a: tier rename to Core/Established/Standard + risk_score and single_source data quality fixes via transformer
Add scripts/transform_dataset.py (deterministic, seed 42): renames tiers,
varies risk_score (was saturated at 100), flags ~20% single_source_risk (was 0),
and recomputes composite_score/calculated_tier/tier_mismatch. Rename tier
literals across TS + Python (NOT the Kraljic 'Strategic' quadrant). Update docs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/procurement_data.xlsx
+++ b/data/raw/procurement_data.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Purchases" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SupplierMetrics" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Suppliers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Purchases" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SupplierMetrics" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,24 +27,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -59,11 +48,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,42 +417,34 @@
   </sheetPr>
   <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>supplier_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>supplier_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>country</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>product_description</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>tier</t>
         </is>
@@ -500,7 +478,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -532,7 +510,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -564,7 +542,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -596,7 +574,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -628,7 +606,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -660,7 +638,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -692,7 +670,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -724,7 +702,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -756,7 +734,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -788,7 +766,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -820,7 +798,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -852,7 +830,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -884,7 +862,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -916,7 +894,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -948,7 +926,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -980,7 +958,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1012,7 +990,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1022,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1054,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1086,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1118,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1150,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1182,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1214,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1246,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1278,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1310,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1342,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1374,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1406,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1438,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1470,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1502,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1534,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1566,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1598,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1630,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1662,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1694,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1726,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1758,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1790,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1822,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1854,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1886,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1918,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1950,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -2004,7 +1982,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2014,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2046,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2078,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2110,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2142,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -2196,7 +2174,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2206,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -2245,138 +2223,114 @@
   </sheetPr>
   <dimension ref="A1:V641"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
-    <col width="25" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
-    <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>po_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>supplier_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>supplier_name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>item_description</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>unit_price_usd</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>total_value_usd</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>pr_date</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>po_date</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>delivery_date</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>invoice_date</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>payment_date</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>pr_to_po_days</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>po_to_delivery_days</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>delivery_to_invoice_days</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>invoice_to_payment_days</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>total_cycle_days</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>on_time_delivery</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>three_way_match_pass</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>automation_period</t>
         </is>
@@ -61275,162 +61229,134 @@
   </sheetPr>
   <dimension ref="A1:Z56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="24" customWidth="1" min="15" max="15"/>
-    <col width="23" customWidth="1" min="16" max="16"/>
-    <col width="24" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="15" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="15" customWidth="1" min="21" max="21"/>
-    <col width="15" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="17" customWidth="1" min="24" max="24"/>
-    <col width="17" customWidth="1" min="25" max="25"/>
-    <col width="15" customWidth="1" min="26" max="26"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>supplier_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>supplier_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>country</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>product_description</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>tier</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>total_spend_usd</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>num_pos</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>avg_po_value_usd</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>avg_lead_time_days</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>avg_cycle_time_days</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>on_time_delivery_pct</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>three_way_match_pct</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>defect_rate_pct</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>complaint_count_annual</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>rfx_response_rate_pct</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>avg_response_time_days</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>single_source_risk</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>quality_score</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>delivery_score</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>service_score</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>process_score</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>risk_score</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>composite_score</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>calculated_tier</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>tier_mismatch</t>
         </is>
@@ -61464,7 +61390,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -61516,14 +61442,14 @@
         <v>84.62</v>
       </c>
       <c r="W2" t="n">
-        <v>100</v>
+        <v>41.31</v>
       </c>
       <c r="X2" t="n">
-        <v>87.15000000000001</v>
+        <v>78.79000000000001</v>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z2" t="b">
@@ -61558,7 +61484,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -61610,18 +61536,18 @@
         <v>78.56999999999999</v>
       </c>
       <c r="W3" t="n">
-        <v>100</v>
+        <v>18.74</v>
       </c>
       <c r="X3" t="n">
-        <v>86.23999999999999</v>
+        <v>74.67</v>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -61652,7 +61578,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -61704,14 +61630,14 @@
         <v>67.73999999999999</v>
       </c>
       <c r="W4" t="n">
-        <v>100</v>
+        <v>47.51</v>
       </c>
       <c r="X4" t="n">
-        <v>83.76000000000001</v>
+        <v>76</v>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z4" t="b">
@@ -61746,7 +61672,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -61798,14 +61724,14 @@
         <v>88.45999999999999</v>
       </c>
       <c r="W5" t="n">
-        <v>100</v>
+        <v>72.84999999999999</v>
       </c>
       <c r="X5" t="n">
-        <v>80.83</v>
+        <v>77.55</v>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z5" t="b">
@@ -61840,7 +61766,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -61892,14 +61818,14 @@
         <v>69.23</v>
       </c>
       <c r="W6" t="n">
-        <v>100</v>
+        <v>30.1</v>
       </c>
       <c r="X6" t="n">
-        <v>73.58</v>
+        <v>64.25</v>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z6" t="b">
@@ -61934,7 +61860,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -61986,18 +61912,18 @@
         <v>73.33</v>
       </c>
       <c r="W7" t="n">
-        <v>100</v>
+        <v>33.6</v>
       </c>
       <c r="X7" t="n">
-        <v>78.19</v>
+        <v>69.02</v>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -62028,7 +61954,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -62080,14 +62006,14 @@
         <v>100</v>
       </c>
       <c r="W8" t="n">
-        <v>100</v>
+        <v>58.81</v>
       </c>
       <c r="X8" t="n">
-        <v>72.17</v>
+        <v>69.08</v>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z8" t="b">
@@ -62122,7 +62048,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -62174,14 +62100,14 @@
         <v>91.67</v>
       </c>
       <c r="W9" t="n">
-        <v>100</v>
+        <v>56.26</v>
       </c>
       <c r="X9" t="n">
-        <v>74.76000000000001</v>
+        <v>69.59</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z9" t="b">
@@ -62216,7 +62142,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -62268,18 +62194,18 @@
         <v>63.64</v>
       </c>
       <c r="W10" t="n">
-        <v>100</v>
+        <v>48.16</v>
       </c>
       <c r="X10" t="n">
-        <v>78.18000000000001</v>
+        <v>71.72</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -62310,7 +62236,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -62362,18 +62288,18 @@
         <v>73.91</v>
       </c>
       <c r="W11" t="n">
-        <v>100</v>
+        <v>44.97</v>
       </c>
       <c r="X11" t="n">
-        <v>80.03</v>
+        <v>72.2</v>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -62404,7 +62330,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -62456,14 +62382,14 @@
         <v>75</v>
       </c>
       <c r="W12" t="n">
-        <v>100</v>
+        <v>71.25</v>
       </c>
       <c r="X12" t="n">
-        <v>79.83</v>
+        <v>77.14</v>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z12" t="b">
@@ -62498,7 +62424,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -62535,7 +62461,7 @@
         <v>4.37</v>
       </c>
       <c r="R13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" t="n">
         <v>62.48</v>
@@ -62550,14 +62476,14 @@
         <v>77.78</v>
       </c>
       <c r="W13" t="n">
-        <v>100</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="X13" t="n">
-        <v>69.29000000000001</v>
+        <v>68.41</v>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z13" t="b">
@@ -62592,7 +62518,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -62644,14 +62570,14 @@
         <v>66.67</v>
       </c>
       <c r="W14" t="n">
-        <v>100</v>
+        <v>56.88</v>
       </c>
       <c r="X14" t="n">
-        <v>71.98999999999999</v>
+        <v>67.51000000000001</v>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z14" t="b">
@@ -62686,7 +62612,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -62723,7 +62649,7 @@
         <v>1.26</v>
       </c>
       <c r="R15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S15" t="n">
         <v>89.18000000000001</v>
@@ -62738,14 +62664,14 @@
         <v>55.17</v>
       </c>
       <c r="W15" t="n">
-        <v>100</v>
+        <v>67.05</v>
       </c>
       <c r="X15" t="n">
-        <v>83.11</v>
+        <v>78.70999999999999</v>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z15" t="b">
@@ -62780,7 +62706,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -62832,14 +62758,14 @@
         <v>73.33</v>
       </c>
       <c r="W16" t="n">
-        <v>100</v>
+        <v>67.29000000000001</v>
       </c>
       <c r="X16" t="n">
-        <v>81.33</v>
+        <v>76.66</v>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z16" t="b">
@@ -62874,7 +62800,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -62926,14 +62852,14 @@
         <v>42.86</v>
       </c>
       <c r="W17" t="n">
-        <v>100</v>
+        <v>34.47</v>
       </c>
       <c r="X17" t="n">
-        <v>67.84</v>
+        <v>58.95</v>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z17" t="b">
@@ -62968,7 +62894,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -63005,7 +62931,7 @@
         <v>0.68</v>
       </c>
       <c r="R18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S18" t="n">
         <v>81.20999999999999</v>
@@ -63020,14 +62946,14 @@
         <v>87.5</v>
       </c>
       <c r="W18" t="n">
-        <v>100</v>
+        <v>50.48</v>
       </c>
       <c r="X18" t="n">
-        <v>85.73999999999999</v>
+        <v>79.25</v>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z18" t="b">
@@ -63062,7 +62988,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -63099,7 +63025,7 @@
         <v>2.98</v>
       </c>
       <c r="R19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S19" t="n">
         <v>74.19</v>
@@ -63114,14 +63040,14 @@
         <v>53.33</v>
       </c>
       <c r="W19" t="n">
-        <v>100</v>
+        <v>32.57</v>
       </c>
       <c r="X19" t="n">
-        <v>72.39</v>
+        <v>63.57</v>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z19" t="b">
@@ -63156,7 +63082,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -63208,14 +63134,14 @@
         <v>50</v>
       </c>
       <c r="W20" t="n">
-        <v>100</v>
+        <v>71.72</v>
       </c>
       <c r="X20" t="n">
-        <v>71.36</v>
+        <v>68.97</v>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z20" t="b">
@@ -63250,7 +63176,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -63302,14 +63228,14 @@
         <v>84.62</v>
       </c>
       <c r="W21" t="n">
-        <v>100</v>
+        <v>64.08</v>
       </c>
       <c r="X21" t="n">
-        <v>69.17</v>
+        <v>65.62</v>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z21" t="b">
@@ -63344,7 +63270,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -63396,14 +63322,14 @@
         <v>87.5</v>
       </c>
       <c r="W22" t="n">
-        <v>100</v>
+        <v>64.65000000000001</v>
       </c>
       <c r="X22" t="n">
-        <v>72.40000000000001</v>
+        <v>69.05</v>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z22" t="b">
@@ -63438,7 +63364,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -63490,14 +63416,14 @@
         <v>50</v>
       </c>
       <c r="W23" t="n">
-        <v>100</v>
+        <v>52.73</v>
       </c>
       <c r="X23" t="n">
-        <v>63.95</v>
+        <v>58.57</v>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z23" t="b">
@@ -63532,7 +63458,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -63584,14 +63510,14 @@
         <v>77.78</v>
       </c>
       <c r="W24" t="n">
-        <v>100</v>
+        <v>65.06</v>
       </c>
       <c r="X24" t="n">
-        <v>84.73999999999999</v>
+        <v>79.98</v>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z24" t="b">
@@ -63626,7 +63552,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -63678,14 +63604,14 @@
         <v>96.15000000000001</v>
       </c>
       <c r="W25" t="n">
-        <v>100</v>
+        <v>48.76</v>
       </c>
       <c r="X25" t="n">
-        <v>82.62</v>
+        <v>76.22</v>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z25" t="b">
@@ -63720,7 +63646,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -63772,18 +63698,18 @@
         <v>54.84</v>
       </c>
       <c r="W26" t="n">
-        <v>100</v>
+        <v>37.34</v>
       </c>
       <c r="X26" t="n">
-        <v>80.68000000000001</v>
+        <v>71.64</v>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -63814,7 +63740,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -63866,18 +63792,18 @@
         <v>100</v>
       </c>
       <c r="W27" t="n">
-        <v>100</v>
+        <v>46.27</v>
       </c>
       <c r="X27" t="n">
-        <v>77.14</v>
+        <v>70.84</v>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -63908,7 +63834,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -63960,14 +63886,14 @@
         <v>66.67</v>
       </c>
       <c r="W28" t="n">
-        <v>100</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="X28" t="n">
-        <v>72.20999999999999</v>
+        <v>69.75</v>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z28" t="b">
@@ -64002,7 +63928,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -64039,7 +63965,7 @@
         <v>13.76</v>
       </c>
       <c r="R29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S29" t="n">
         <v>58.39</v>
@@ -64054,14 +63980,14 @@
         <v>100</v>
       </c>
       <c r="W29" t="n">
-        <v>100</v>
+        <v>59.31</v>
       </c>
       <c r="X29" t="n">
-        <v>71.28</v>
+        <v>67.26000000000001</v>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z29" t="b">
@@ -64096,7 +64022,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G30" t="n">
@@ -64148,18 +64074,18 @@
         <v>100</v>
       </c>
       <c r="W30" t="n">
-        <v>100</v>
+        <v>57.33</v>
       </c>
       <c r="X30" t="n">
-        <v>59.87</v>
+        <v>56.68</v>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -64190,7 +64116,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -64242,18 +64168,18 @@
         <v>81.81999999999999</v>
       </c>
       <c r="W31" t="n">
-        <v>100</v>
+        <v>63.49</v>
       </c>
       <c r="X31" t="n">
-        <v>79.93000000000001</v>
+        <v>74.77</v>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -64284,7 +64210,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G32" t="n">
@@ -64336,14 +64262,14 @@
         <v>77.78</v>
       </c>
       <c r="W32" t="n">
-        <v>100</v>
+        <v>90.34999999999999</v>
       </c>
       <c r="X32" t="n">
-        <v>76.87</v>
+        <v>76.22</v>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z32" t="b">
@@ -64378,7 +64304,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G33" t="n">
@@ -64415,7 +64341,7 @@
         <v>2.28</v>
       </c>
       <c r="R33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S33" t="n">
         <v>53.61</v>
@@ -64430,14 +64356,14 @@
         <v>57.14</v>
       </c>
       <c r="W33" t="n">
-        <v>100</v>
+        <v>56.77</v>
       </c>
       <c r="X33" t="n">
-        <v>64.11</v>
+        <v>59.95</v>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z33" t="b">
@@ -64472,7 +64398,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -64524,14 +64450,14 @@
         <v>70</v>
       </c>
       <c r="W34" t="n">
-        <v>100</v>
+        <v>61.66</v>
       </c>
       <c r="X34" t="n">
-        <v>56.73</v>
+        <v>54.28</v>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="Z34" t="b">
@@ -64566,7 +64492,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G35" t="n">
@@ -64618,14 +64544,14 @@
         <v>87.5</v>
       </c>
       <c r="W35" t="n">
-        <v>100</v>
+        <v>59.27</v>
       </c>
       <c r="X35" t="n">
-        <v>64.48999999999999</v>
+        <v>60.99</v>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z35" t="b">
@@ -64660,7 +64586,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G36" t="n">
@@ -64712,18 +64638,18 @@
         <v>50</v>
       </c>
       <c r="W36" t="n">
-        <v>100</v>
+        <v>70.05</v>
       </c>
       <c r="X36" t="n">
-        <v>56.93</v>
+        <v>56.61</v>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -64754,7 +64680,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G37" t="n">
@@ -64806,14 +64732,14 @@
         <v>86.67</v>
       </c>
       <c r="W37" t="n">
-        <v>100</v>
+        <v>88.16</v>
       </c>
       <c r="X37" t="n">
-        <v>71.2</v>
+        <v>70.58</v>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z37" t="b">
@@ -64848,7 +64774,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G38" t="n">
@@ -64900,14 +64826,14 @@
         <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>100</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="X38" t="n">
-        <v>47.96</v>
+        <v>46.07</v>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="Z38" t="b">
@@ -64942,7 +64868,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G39" t="n">
@@ -64994,18 +64920,18 @@
         <v>85.70999999999999</v>
       </c>
       <c r="W39" t="n">
-        <v>100</v>
+        <v>49.83</v>
       </c>
       <c r="X39" t="n">
-        <v>78</v>
+        <v>71.3</v>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -65036,7 +64962,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G40" t="n">
@@ -65088,14 +65014,14 @@
         <v>100</v>
       </c>
       <c r="W40" t="n">
-        <v>100</v>
+        <v>59.14</v>
       </c>
       <c r="X40" t="n">
-        <v>62.54</v>
+        <v>59.19</v>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z40" t="b">
@@ -65130,7 +65056,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G41" t="n">
@@ -65182,14 +65108,14 @@
         <v>85.70999999999999</v>
       </c>
       <c r="W41" t="n">
-        <v>100</v>
+        <v>76.68000000000001</v>
       </c>
       <c r="X41" t="n">
-        <v>71.41</v>
+        <v>69.03</v>
       </c>
       <c r="Y41" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z41" t="b">
@@ -65224,7 +65150,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G42" t="n">
@@ -65261,7 +65187,7 @@
         <v>1.09</v>
       </c>
       <c r="R42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S42" t="n">
         <v>69.86</v>
@@ -65276,14 +65202,14 @@
         <v>90.91</v>
       </c>
       <c r="W42" t="n">
-        <v>100</v>
+        <v>78.33</v>
       </c>
       <c r="X42" t="n">
-        <v>73.31</v>
+        <v>71.56</v>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z42" t="b">
@@ -65318,7 +65244,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G43" t="n">
@@ -65355,7 +65281,7 @@
         <v>6.23</v>
       </c>
       <c r="R43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S43" t="n">
         <v>49.12</v>
@@ -65370,14 +65296,14 @@
         <v>100</v>
       </c>
       <c r="W43" t="n">
-        <v>100</v>
+        <v>65.77</v>
       </c>
       <c r="X43" t="n">
-        <v>72.28</v>
+        <v>69.69</v>
       </c>
       <c r="Y43" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z43" t="b">
@@ -65412,7 +65338,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="G44" t="n">
@@ -65464,18 +65390,18 @@
         <v>80.65000000000001</v>
       </c>
       <c r="W44" t="n">
-        <v>100</v>
+        <v>45.76</v>
       </c>
       <c r="X44" t="n">
-        <v>80.87</v>
+        <v>73.06</v>
       </c>
       <c r="Y44" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -65506,7 +65432,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G45" t="n">
@@ -65558,14 +65484,14 @@
         <v>100</v>
       </c>
       <c r="W45" t="n">
-        <v>100</v>
+        <v>65.98</v>
       </c>
       <c r="X45" t="n">
-        <v>81.5</v>
+        <v>77.33</v>
       </c>
       <c r="Y45" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z45" t="b">
@@ -65600,7 +65526,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G46" t="n">
@@ -65652,14 +65578,14 @@
         <v>66.67</v>
       </c>
       <c r="W46" t="n">
-        <v>100</v>
+        <v>63.84</v>
       </c>
       <c r="X46" t="n">
-        <v>74.25</v>
+        <v>69.43000000000001</v>
       </c>
       <c r="Y46" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z46" t="b">
@@ -65694,7 +65620,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G47" t="n">
@@ -65746,18 +65672,18 @@
         <v>93.33</v>
       </c>
       <c r="W47" t="n">
-        <v>100</v>
+        <v>56.82</v>
       </c>
       <c r="X47" t="n">
-        <v>78.86</v>
+        <v>74.14</v>
       </c>
       <c r="Y47" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z47" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -65788,7 +65714,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G48" t="n">
@@ -65840,14 +65766,14 @@
         <v>0</v>
       </c>
       <c r="W48" t="n">
-        <v>100</v>
+        <v>68.69</v>
       </c>
       <c r="X48" t="n">
-        <v>52.39</v>
+        <v>49.24</v>
       </c>
       <c r="Y48" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="Z48" t="b">
@@ -65882,7 +65808,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G49" t="n">
@@ -65934,14 +65860,14 @@
         <v>100</v>
       </c>
       <c r="W49" t="n">
-        <v>100</v>
+        <v>59.99</v>
       </c>
       <c r="X49" t="n">
-        <v>77.31</v>
+        <v>73.68000000000001</v>
       </c>
       <c r="Y49" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z49" t="b">
@@ -65976,7 +65902,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G50" t="n">
@@ -66028,14 +65954,14 @@
         <v>33.33</v>
       </c>
       <c r="W50" t="n">
-        <v>100</v>
+        <v>71.19</v>
       </c>
       <c r="X50" t="n">
-        <v>54.96</v>
+        <v>54.36</v>
       </c>
       <c r="Y50" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="Z50" t="b">
@@ -66070,7 +65996,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G51" t="n">
@@ -66122,14 +66048,14 @@
         <v>83.33</v>
       </c>
       <c r="W51" t="n">
-        <v>100</v>
+        <v>51.16</v>
       </c>
       <c r="X51" t="n">
-        <v>69.48999999999999</v>
+        <v>64.84</v>
       </c>
       <c r="Y51" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z51" t="b">
@@ -66164,7 +66090,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="G52" t="n">
@@ -66201,7 +66127,7 @@
         <v>0.95</v>
       </c>
       <c r="R52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S52" t="n">
         <v>70.06999999999999</v>
@@ -66216,14 +66142,14 @@
         <v>100</v>
       </c>
       <c r="W52" t="n">
-        <v>100</v>
+        <v>58.15</v>
       </c>
       <c r="X52" t="n">
-        <v>82.98999999999999</v>
+        <v>78.20999999999999</v>
       </c>
       <c r="Y52" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z52" t="b">
@@ -66258,7 +66184,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G53" t="n">
@@ -66295,7 +66221,7 @@
         <v>2.23</v>
       </c>
       <c r="R53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S53" t="n">
         <v>22.41</v>
@@ -66310,14 +66236,14 @@
         <v>100</v>
       </c>
       <c r="W53" t="n">
-        <v>100</v>
+        <v>67.3</v>
       </c>
       <c r="X53" t="n">
-        <v>60.2</v>
+        <v>59.17</v>
       </c>
       <c r="Y53" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z53" t="b">
@@ -66352,7 +66278,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G54" t="n">
@@ -66404,14 +66330,14 @@
         <v>100</v>
       </c>
       <c r="W54" t="n">
-        <v>100</v>
+        <v>26.75</v>
       </c>
       <c r="X54" t="n">
-        <v>84.02</v>
+        <v>74.8</v>
       </c>
       <c r="Y54" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z54" t="b">
@@ -66446,7 +66372,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G55" t="n">
@@ -66498,14 +66424,14 @@
         <v>0</v>
       </c>
       <c r="W55" t="n">
-        <v>100</v>
+        <v>44.21</v>
       </c>
       <c r="X55" t="n">
-        <v>58.57</v>
+        <v>52.19</v>
       </c>
       <c r="Y55" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="Z55" t="b">
@@ -66540,7 +66466,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="G56" t="n">
@@ -66577,7 +66503,7 @@
         <v>3.54</v>
       </c>
       <c r="R56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S56" t="n">
         <v>42.08</v>
@@ -66592,14 +66518,14 @@
         <v>100</v>
       </c>
       <c r="W56" t="n">
-        <v>100</v>
+        <v>50.49</v>
       </c>
       <c r="X56" t="n">
-        <v>66.48</v>
+        <v>61.95</v>
       </c>
       <c r="Y56" t="inlineStr">
         <is>
-          <t>Preferred</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z56" t="b">

</xml_diff>

<commit_message>
Methodology rebuild — all sub-scores derived from raw data with fixed bounds, risk score fully deterministic, tier mismatch badge softened to diagnostic
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/procurement_data.xlsx
+++ b/data/raw/procurement_data.xlsx
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,32 +431,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>supplier_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>supplier_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>country</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>product_description</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>tier</t>
         </is>
@@ -2225,107 +2237,107 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>po_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>supplier_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>supplier_name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>item_description</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>unit_price_usd</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>total_value_usd</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>pr_date</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>po_date</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>delivery_date</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>invoice_date</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>payment_date</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>pr_to_po_days</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>po_to_delivery_days</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>delivery_to_invoice_days</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>invoice_to_payment_days</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>total_cycle_days</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>on_time_delivery</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>three_way_match_pass</t>
         </is>
@@ -58026,132 +58038,132 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>supplier_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>supplier_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>country</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>product_description</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>tier</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>total_spend_usd</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>num_pos</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>avg_po_value_usd</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>avg_lead_time_days</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>avg_cycle_time_days</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>on_time_delivery_pct</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>three_way_match_pct</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>defect_rate_pct</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>complaint_count_annual</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>rfx_response_rate_pct</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>avg_response_time_days</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>single_source_risk</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>quality_score</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>delivery_score</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>service_score</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>process_score</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>risk_score</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>composite_score</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>calculated_tier</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>tier_mismatch</t>
         </is>
@@ -58225,22 +58237,22 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>91.01000000000001</v>
+        <v>92.84999999999999</v>
       </c>
       <c r="T2" t="n">
-        <v>75.51000000000001</v>
+        <v>85.95999999999999</v>
       </c>
       <c r="U2" t="n">
-        <v>93.61</v>
+        <v>90.31999999999999</v>
       </c>
       <c r="V2" t="n">
         <v>84.62</v>
       </c>
       <c r="W2" t="n">
-        <v>41.31</v>
+        <v>100</v>
       </c>
       <c r="X2" t="n">
-        <v>78.79000000000001</v>
+        <v>90.17</v>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
@@ -58319,30 +58331,30 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>87.63</v>
+        <v>90.15000000000001</v>
       </c>
       <c r="T3" t="n">
-        <v>78.43000000000001</v>
+        <v>88.48</v>
       </c>
       <c r="U3" t="n">
-        <v>97.55</v>
+        <v>94.16</v>
       </c>
       <c r="V3" t="n">
         <v>78.56999999999999</v>
       </c>
       <c r="W3" t="n">
-        <v>18.74</v>
+        <v>97</v>
       </c>
       <c r="X3" t="n">
-        <v>74.67</v>
+        <v>89.05</v>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -58413,22 +58425,22 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>97.70999999999999</v>
+        <v>96.95</v>
       </c>
       <c r="T4" t="n">
-        <v>70.44</v>
+        <v>82.44</v>
       </c>
       <c r="U4" t="n">
-        <v>88.56</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="V4" t="n">
         <v>67.73999999999999</v>
       </c>
       <c r="W4" t="n">
-        <v>47.51</v>
+        <v>100</v>
       </c>
       <c r="X4" t="n">
-        <v>76</v>
+        <v>86.51000000000001</v>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
@@ -58507,22 +58519,22 @@
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>84.08</v>
+        <v>87.34999999999999</v>
       </c>
       <c r="T5" t="n">
-        <v>52.49</v>
+        <v>75.8</v>
       </c>
       <c r="U5" t="n">
-        <v>98.59</v>
+        <v>95.17</v>
       </c>
       <c r="V5" t="n">
         <v>88.45999999999999</v>
       </c>
       <c r="W5" t="n">
-        <v>72.84999999999999</v>
+        <v>54</v>
       </c>
       <c r="X5" t="n">
-        <v>77.55</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
@@ -58601,22 +58613,22 @@
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>76.86</v>
+        <v>82.3</v>
       </c>
       <c r="T6" t="n">
-        <v>49.67</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="U6" t="n">
-        <v>95.06999999999999</v>
+        <v>92.20999999999999</v>
       </c>
       <c r="V6" t="n">
         <v>69.23</v>
       </c>
       <c r="W6" t="n">
-        <v>30.1</v>
+        <v>51</v>
       </c>
       <c r="X6" t="n">
-        <v>64.25</v>
+        <v>74</v>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
@@ -58695,30 +58707,30 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>84.2</v>
+        <v>88.05</v>
       </c>
       <c r="T7" t="n">
-        <v>56.91</v>
+        <v>79.11</v>
       </c>
       <c r="U7" t="n">
-        <v>93.56</v>
+        <v>90.81999999999999</v>
       </c>
       <c r="V7" t="n">
         <v>73.33</v>
       </c>
       <c r="W7" t="n">
-        <v>33.6</v>
+        <v>57</v>
       </c>
       <c r="X7" t="n">
-        <v>69.02</v>
+        <v>78.63</v>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -58789,30 +58801,30 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>38.24</v>
+        <v>56.15</v>
       </c>
       <c r="T8" t="n">
-        <v>73.44</v>
+        <v>84.28</v>
       </c>
       <c r="U8" t="n">
-        <v>82.27</v>
+        <v>80.92</v>
       </c>
       <c r="V8" t="n">
         <v>100</v>
       </c>
       <c r="W8" t="n">
-        <v>58.81</v>
+        <v>79</v>
       </c>
       <c r="X8" t="n">
-        <v>69.08</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -58883,30 +58895,30 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>72.23</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="T9" t="n">
-        <v>53.7</v>
+        <v>77.23</v>
       </c>
       <c r="U9" t="n">
-        <v>75.56999999999999</v>
+        <v>72.29000000000001</v>
       </c>
       <c r="V9" t="n">
         <v>91.67</v>
       </c>
       <c r="W9" t="n">
-        <v>56.26</v>
+        <v>54</v>
       </c>
       <c r="X9" t="n">
-        <v>69.59</v>
+        <v>76.61</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -58977,30 +58989,30 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>73.7</v>
+        <v>81</v>
       </c>
       <c r="T10" t="n">
-        <v>79.45999999999999</v>
+        <v>89.66</v>
       </c>
       <c r="U10" t="n">
-        <v>89.88</v>
+        <v>87.45999999999999</v>
       </c>
       <c r="V10" t="n">
         <v>63.64</v>
       </c>
       <c r="W10" t="n">
-        <v>48.16</v>
+        <v>94</v>
       </c>
       <c r="X10" t="n">
-        <v>71.72</v>
+        <v>82.61</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -59071,30 +59083,30 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>91.47</v>
+        <v>92.5</v>
       </c>
       <c r="T11" t="n">
-        <v>53.97</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="U11" t="n">
-        <v>95.41</v>
+        <v>92.81999999999999</v>
       </c>
       <c r="V11" t="n">
         <v>73.91</v>
       </c>
       <c r="W11" t="n">
-        <v>44.97</v>
+        <v>57</v>
       </c>
       <c r="X11" t="n">
-        <v>72.2</v>
+        <v>79.69</v>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -59165,22 +59177,22 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>67.43000000000001</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="T12" t="n">
-        <v>82.3</v>
+        <v>92.18000000000001</v>
       </c>
       <c r="U12" t="n">
-        <v>93.48999999999999</v>
+        <v>90.41</v>
       </c>
       <c r="V12" t="n">
         <v>75</v>
       </c>
       <c r="W12" t="n">
-        <v>71.25</v>
+        <v>88</v>
       </c>
       <c r="X12" t="n">
-        <v>77.14</v>
+        <v>83.78</v>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
@@ -59259,22 +59271,22 @@
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>62.48</v>
+        <v>73.5</v>
       </c>
       <c r="T13" t="n">
-        <v>49.16</v>
+        <v>74.44</v>
       </c>
       <c r="U13" t="n">
-        <v>84.67</v>
+        <v>80.64</v>
       </c>
       <c r="V13" t="n">
         <v>77.78</v>
       </c>
       <c r="W13" t="n">
-        <v>81.59999999999999</v>
+        <v>21</v>
       </c>
       <c r="X13" t="n">
-        <v>68.41</v>
+        <v>67.79000000000001</v>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
@@ -59353,26 +59365,26 @@
         <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>60.4</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="T14" t="n">
-        <v>83.02</v>
+        <v>92.5</v>
       </c>
       <c r="U14" t="n">
-        <v>65.23</v>
+        <v>62.35</v>
       </c>
       <c r="V14" t="n">
         <v>66.67</v>
       </c>
       <c r="W14" t="n">
-        <v>56.88</v>
+        <v>88</v>
       </c>
       <c r="X14" t="n">
-        <v>67.51000000000001</v>
+        <v>76.91</v>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z14" t="b">
@@ -59447,22 +59459,22 @@
         <v>1</v>
       </c>
       <c r="S15" t="n">
-        <v>89.18000000000001</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="T15" t="n">
-        <v>83.15000000000001</v>
+        <v>92.56</v>
       </c>
       <c r="U15" t="n">
-        <v>96.90000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="V15" t="n">
         <v>55.17</v>
       </c>
       <c r="W15" t="n">
-        <v>67.05</v>
+        <v>67</v>
       </c>
       <c r="X15" t="n">
-        <v>78.70999999999999</v>
+        <v>81.05</v>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
@@ -59541,22 +59553,22 @@
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>95.18000000000001</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="T16" t="n">
-        <v>56.16</v>
+        <v>78.77</v>
       </c>
       <c r="U16" t="n">
-        <v>93.78</v>
+        <v>91.38</v>
       </c>
       <c r="V16" t="n">
         <v>73.33</v>
       </c>
       <c r="W16" t="n">
-        <v>67.29000000000001</v>
+        <v>76</v>
       </c>
       <c r="X16" t="n">
-        <v>76.66</v>
+        <v>83.31999999999999</v>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
@@ -59635,22 +59647,22 @@
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>81.3</v>
+        <v>85.65000000000001</v>
       </c>
       <c r="T17" t="n">
-        <v>63.07</v>
+        <v>75.72</v>
       </c>
       <c r="U17" t="n">
-        <v>60.75</v>
+        <v>61.82</v>
       </c>
       <c r="V17" t="n">
         <v>42.86</v>
       </c>
       <c r="W17" t="n">
-        <v>34.47</v>
+        <v>94</v>
       </c>
       <c r="X17" t="n">
-        <v>58.95</v>
+        <v>72.29000000000001</v>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
@@ -59729,22 +59741,22 @@
         <v>1</v>
       </c>
       <c r="S18" t="n">
-        <v>81.20999999999999</v>
+        <v>86.84999999999999</v>
       </c>
       <c r="T18" t="n">
-        <v>76.41</v>
+        <v>86.09</v>
       </c>
       <c r="U18" t="n">
-        <v>98.5</v>
+        <v>95.59</v>
       </c>
       <c r="V18" t="n">
         <v>87.5</v>
       </c>
       <c r="W18" t="n">
-        <v>50.48</v>
+        <v>70</v>
       </c>
       <c r="X18" t="n">
-        <v>79.25</v>
+        <v>85.56999999999999</v>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
@@ -59823,22 +59835,22 @@
         <v>1</v>
       </c>
       <c r="S19" t="n">
-        <v>74.19</v>
+        <v>81.3</v>
       </c>
       <c r="T19" t="n">
-        <v>67.87</v>
+        <v>80.22</v>
       </c>
       <c r="U19" t="n">
-        <v>83.36</v>
+        <v>81.14</v>
       </c>
       <c r="V19" t="n">
         <v>53.33</v>
       </c>
       <c r="W19" t="n">
-        <v>32.57</v>
+        <v>64</v>
       </c>
       <c r="X19" t="n">
-        <v>63.57</v>
+        <v>72.81999999999999</v>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
@@ -59917,30 +59929,30 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>62.77</v>
+        <v>73.05</v>
       </c>
       <c r="T20" t="n">
-        <v>81.13</v>
+        <v>91.67</v>
       </c>
       <c r="U20" t="n">
-        <v>81.61</v>
+        <v>81.68000000000001</v>
       </c>
       <c r="V20" t="n">
         <v>50</v>
       </c>
       <c r="W20" t="n">
-        <v>71.72</v>
+        <v>88</v>
       </c>
       <c r="X20" t="n">
-        <v>68.97</v>
+        <v>76.63</v>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -60011,22 +60023,22 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>63.33</v>
+        <v>74.65000000000001</v>
       </c>
       <c r="T21" t="n">
-        <v>43.33</v>
+        <v>68.53</v>
       </c>
       <c r="U21" t="n">
-        <v>82.78</v>
+        <v>83.08</v>
       </c>
       <c r="V21" t="n">
         <v>84.62</v>
       </c>
       <c r="W21" t="n">
-        <v>64.08</v>
+        <v>54</v>
       </c>
       <c r="X21" t="n">
-        <v>65.62</v>
+        <v>73.28</v>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
@@ -60105,30 +60117,30 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>60.92</v>
+        <v>72.55</v>
       </c>
       <c r="T22" t="n">
-        <v>61.79</v>
+        <v>83.12</v>
       </c>
       <c r="U22" t="n">
-        <v>74.5</v>
+        <v>75.02</v>
       </c>
       <c r="V22" t="n">
         <v>87.5</v>
       </c>
       <c r="W22" t="n">
-        <v>64.65000000000001</v>
+        <v>51</v>
       </c>
       <c r="X22" t="n">
-        <v>69.05</v>
+        <v>75.31999999999999</v>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -60199,22 +60211,22 @@
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>65.62</v>
+        <v>76.05</v>
       </c>
       <c r="T23" t="n">
-        <v>59.43</v>
+        <v>82.08</v>
       </c>
       <c r="U23" t="n">
-        <v>62.68</v>
+        <v>61.62</v>
       </c>
       <c r="V23" t="n">
         <v>50</v>
       </c>
       <c r="W23" t="n">
-        <v>52.73</v>
+        <v>54</v>
       </c>
       <c r="X23" t="n">
-        <v>58.57</v>
+        <v>66.88</v>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
@@ -60293,22 +60305,22 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>90.36</v>
+        <v>92.45</v>
       </c>
       <c r="T24" t="n">
-        <v>72.38</v>
+        <v>83.15000000000001</v>
       </c>
       <c r="U24" t="n">
-        <v>93.23</v>
+        <v>89.63</v>
       </c>
       <c r="V24" t="n">
         <v>77.78</v>
       </c>
       <c r="W24" t="n">
-        <v>65.06</v>
+        <v>100</v>
       </c>
       <c r="X24" t="n">
-        <v>79.98</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
@@ -60387,22 +60399,22 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>74.31999999999999</v>
+        <v>80.75</v>
       </c>
       <c r="T25" t="n">
-        <v>67.48</v>
+        <v>79.19</v>
       </c>
       <c r="U25" t="n">
-        <v>94.84</v>
+        <v>91.81999999999999</v>
       </c>
       <c r="V25" t="n">
         <v>96.15000000000001</v>
       </c>
       <c r="W25" t="n">
-        <v>48.76</v>
+        <v>91</v>
       </c>
       <c r="X25" t="n">
-        <v>76.22</v>
+        <v>86.64</v>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
@@ -60481,30 +60493,30 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>92.86</v>
+        <v>93.34999999999999</v>
       </c>
       <c r="T26" t="n">
-        <v>73.89</v>
+        <v>84.87</v>
       </c>
       <c r="U26" t="n">
-        <v>89.23</v>
+        <v>85.33</v>
       </c>
       <c r="V26" t="n">
         <v>54.84</v>
       </c>
       <c r="W26" t="n">
-        <v>37.34</v>
+        <v>97</v>
       </c>
       <c r="X26" t="n">
-        <v>71.64</v>
+        <v>82.87</v>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -60575,30 +60587,30 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>64.84999999999999</v>
+        <v>74.95</v>
       </c>
       <c r="T27" t="n">
-        <v>69.65000000000001</v>
+        <v>81.94</v>
       </c>
       <c r="U27" t="n">
-        <v>68.48</v>
+        <v>70.04000000000001</v>
       </c>
       <c r="V27" t="n">
         <v>100</v>
       </c>
       <c r="W27" t="n">
-        <v>46.27</v>
+        <v>91</v>
       </c>
       <c r="X27" t="n">
-        <v>70.84</v>
+        <v>83.38</v>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -60669,30 +60681,30 @@
         <v>0</v>
       </c>
       <c r="S28" t="n">
-        <v>53.75</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="T28" t="n">
-        <v>82.40000000000001</v>
+        <v>92.22</v>
       </c>
       <c r="U28" t="n">
-        <v>80.98</v>
+        <v>79.84</v>
       </c>
       <c r="V28" t="n">
         <v>66.67</v>
       </c>
       <c r="W28" t="n">
-        <v>68.18000000000001</v>
+        <v>85</v>
       </c>
       <c r="X28" t="n">
-        <v>69.75</v>
+        <v>77.84</v>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -60763,22 +60775,22 @@
         <v>1</v>
       </c>
       <c r="S29" t="n">
-        <v>58.39</v>
+        <v>71</v>
       </c>
       <c r="T29" t="n">
-        <v>82.64</v>
+        <v>92.33</v>
       </c>
       <c r="U29" t="n">
-        <v>20.69</v>
+        <v>19.9</v>
       </c>
       <c r="V29" t="n">
         <v>100</v>
       </c>
       <c r="W29" t="n">
-        <v>59.31</v>
+        <v>61</v>
       </c>
       <c r="X29" t="n">
-        <v>67.26000000000001</v>
+        <v>72.97</v>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
@@ -60857,22 +60869,22 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>35.71</v>
+        <v>57.75</v>
       </c>
       <c r="T30" t="n">
-        <v>49.53</v>
+        <v>63.75</v>
       </c>
       <c r="U30" t="n">
-        <v>45.15</v>
+        <v>49.22</v>
       </c>
       <c r="V30" t="n">
         <v>100</v>
       </c>
       <c r="W30" t="n">
-        <v>57.33</v>
+        <v>94</v>
       </c>
       <c r="X30" t="n">
-        <v>56.68</v>
+        <v>71.86</v>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
@@ -60951,30 +60963,30 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>93.70999999999999</v>
+        <v>94.5</v>
       </c>
       <c r="T31" t="n">
-        <v>44.8</v>
+        <v>69.28</v>
       </c>
       <c r="U31" t="n">
-        <v>95.03</v>
+        <v>91.45999999999999</v>
       </c>
       <c r="V31" t="n">
         <v>81.81999999999999</v>
       </c>
       <c r="W31" t="n">
-        <v>63.49</v>
+        <v>60</v>
       </c>
       <c r="X31" t="n">
-        <v>74.77</v>
+        <v>80.03</v>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -61045,22 +61057,22 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>83.95</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="T32" t="n">
-        <v>55.77</v>
+        <v>80.47</v>
       </c>
       <c r="U32" t="n">
-        <v>81.22</v>
+        <v>78.97</v>
       </c>
       <c r="V32" t="n">
         <v>77.78</v>
       </c>
       <c r="W32" t="n">
-        <v>90.34999999999999</v>
+        <v>73</v>
       </c>
       <c r="X32" t="n">
-        <v>76.22</v>
+        <v>80.44</v>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
@@ -61139,22 +61151,22 @@
         <v>1</v>
       </c>
       <c r="S33" t="n">
-        <v>53.61</v>
+        <v>68.7</v>
       </c>
       <c r="T33" t="n">
-        <v>61.45</v>
+        <v>82.98</v>
       </c>
       <c r="U33" t="n">
-        <v>74.92</v>
+        <v>75.27</v>
       </c>
       <c r="V33" t="n">
         <v>57.14</v>
       </c>
       <c r="W33" t="n">
-        <v>56.77</v>
+        <v>40</v>
       </c>
       <c r="X33" t="n">
-        <v>59.95</v>
+        <v>66.64</v>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
@@ -61233,30 +61245,30 @@
         <v>0</v>
       </c>
       <c r="S34" t="n">
-        <v>34.09</v>
+        <v>55.5</v>
       </c>
       <c r="T34" t="n">
-        <v>45.19</v>
+        <v>67.42</v>
       </c>
       <c r="U34" t="n">
-        <v>74.73</v>
+        <v>75.8</v>
       </c>
       <c r="V34" t="n">
         <v>70</v>
       </c>
       <c r="W34" t="n">
-        <v>61.66</v>
+        <v>48</v>
       </c>
       <c r="X34" t="n">
-        <v>54.28</v>
+        <v>63.3</v>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -61327,22 +61339,22 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>47.86</v>
+        <v>63.3</v>
       </c>
       <c r="T35" t="n">
-        <v>48.1</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="U35" t="n">
-        <v>70.73999999999999</v>
+        <v>70.89</v>
       </c>
       <c r="V35" t="n">
         <v>87.5</v>
       </c>
       <c r="W35" t="n">
-        <v>59.27</v>
+        <v>45</v>
       </c>
       <c r="X35" t="n">
-        <v>60.99</v>
+        <v>68.23</v>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
@@ -61421,22 +61433,22 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>16.49</v>
+        <v>44.1</v>
       </c>
       <c r="T36" t="n">
-        <v>80.19</v>
+        <v>91.25</v>
       </c>
       <c r="U36" t="n">
-        <v>79.54000000000001</v>
+        <v>76.93000000000001</v>
       </c>
       <c r="V36" t="n">
         <v>50</v>
       </c>
       <c r="W36" t="n">
-        <v>70.05</v>
+        <v>85</v>
       </c>
       <c r="X36" t="n">
-        <v>56.61</v>
+        <v>68.13</v>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
@@ -61515,22 +61527,22 @@
         <v>0</v>
       </c>
       <c r="S37" t="n">
-        <v>76.86</v>
+        <v>82.3</v>
       </c>
       <c r="T37" t="n">
-        <v>48.81</v>
+        <v>73.67</v>
       </c>
       <c r="U37" t="n">
-        <v>57.37</v>
+        <v>56.33</v>
       </c>
       <c r="V37" t="n">
         <v>86.67</v>
       </c>
       <c r="W37" t="n">
-        <v>88.16</v>
+        <v>67</v>
       </c>
       <c r="X37" t="n">
-        <v>70.58</v>
+        <v>74.83</v>
       </c>
       <c r="Y37" t="inlineStr">
         <is>
@@ -61609,22 +61621,22 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>53.5</v>
+        <v>66.75</v>
       </c>
       <c r="T38" t="n">
-        <v>50</v>
+        <v>77.92</v>
       </c>
       <c r="U38" t="n">
-        <v>62.71</v>
+        <v>64.98</v>
       </c>
       <c r="V38" t="n">
         <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>71.93000000000001</v>
+        <v>45</v>
       </c>
       <c r="X38" t="n">
-        <v>46.07</v>
+        <v>52.66</v>
       </c>
       <c r="Y38" t="inlineStr">
         <is>
@@ -61703,30 +61715,30 @@
         <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>83.51000000000001</v>
+        <v>87</v>
       </c>
       <c r="T39" t="n">
-        <v>59.04</v>
+        <v>81.91</v>
       </c>
       <c r="U39" t="n">
-        <v>73.63</v>
+        <v>73.23</v>
       </c>
       <c r="V39" t="n">
         <v>85.70999999999999</v>
       </c>
       <c r="W39" t="n">
-        <v>49.83</v>
+        <v>54</v>
       </c>
       <c r="X39" t="n">
-        <v>71.3</v>
+        <v>78.45</v>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -61797,22 +61809,22 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>44.43</v>
+        <v>61.2</v>
       </c>
       <c r="T40" t="n">
-        <v>62.26</v>
+        <v>83.33</v>
       </c>
       <c r="U40" t="n">
-        <v>24.28</v>
+        <v>28.96</v>
       </c>
       <c r="V40" t="n">
         <v>100</v>
       </c>
       <c r="W40" t="n">
-        <v>59.14</v>
+        <v>61</v>
       </c>
       <c r="X40" t="n">
-        <v>59.19</v>
+        <v>69.63</v>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
@@ -61891,22 +61903,22 @@
         <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>77.70999999999999</v>
+        <v>83.45</v>
       </c>
       <c r="T41" t="n">
-        <v>31.4</v>
+        <v>57.74</v>
       </c>
       <c r="U41" t="n">
-        <v>87.38</v>
+        <v>85.31</v>
       </c>
       <c r="V41" t="n">
         <v>85.70999999999999</v>
       </c>
       <c r="W41" t="n">
-        <v>76.68000000000001</v>
+        <v>54</v>
       </c>
       <c r="X41" t="n">
-        <v>69.03</v>
+        <v>73.34</v>
       </c>
       <c r="Y41" t="inlineStr">
         <is>
@@ -61985,22 +61997,22 @@
         <v>1</v>
       </c>
       <c r="S42" t="n">
-        <v>69.86</v>
+        <v>78.65000000000001</v>
       </c>
       <c r="T42" t="n">
-        <v>46.83</v>
+        <v>71.44</v>
       </c>
       <c r="U42" t="n">
-        <v>83.06999999999999</v>
+        <v>83</v>
       </c>
       <c r="V42" t="n">
         <v>90.91</v>
       </c>
       <c r="W42" t="n">
-        <v>78.33</v>
+        <v>24</v>
       </c>
       <c r="X42" t="n">
-        <v>71.56</v>
+        <v>71.75</v>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
@@ -62079,26 +62091,26 @@
         <v>1</v>
       </c>
       <c r="S43" t="n">
-        <v>49.12</v>
+        <v>64.7</v>
       </c>
       <c r="T43" t="n">
-        <v>77.36</v>
+        <v>90</v>
       </c>
       <c r="U43" t="n">
-        <v>54.69</v>
+        <v>54.97</v>
       </c>
       <c r="V43" t="n">
         <v>100</v>
       </c>
       <c r="W43" t="n">
-        <v>65.77</v>
+        <v>58</v>
       </c>
       <c r="X43" t="n">
-        <v>69.69</v>
+        <v>75.62</v>
       </c>
       <c r="Y43" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z43" t="b">
@@ -62173,30 +62185,30 @@
         <v>0</v>
       </c>
       <c r="S44" t="n">
-        <v>93.38</v>
+        <v>94.3</v>
       </c>
       <c r="T44" t="n">
-        <v>53.38</v>
+        <v>75.81</v>
       </c>
       <c r="U44" t="n">
-        <v>89.2</v>
+        <v>87.3</v>
       </c>
       <c r="V44" t="n">
         <v>80.65000000000001</v>
       </c>
       <c r="W44" t="n">
-        <v>45.76</v>
+        <v>60</v>
       </c>
       <c r="X44" t="n">
-        <v>73.06</v>
+        <v>80.75</v>
       </c>
       <c r="Y44" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -62267,22 +62279,22 @@
         <v>0</v>
       </c>
       <c r="S45" t="n">
-        <v>81.26000000000001</v>
+        <v>86.25</v>
       </c>
       <c r="T45" t="n">
-        <v>56.76</v>
+        <v>76.25</v>
       </c>
       <c r="U45" t="n">
-        <v>86.20999999999999</v>
+        <v>85.2</v>
       </c>
       <c r="V45" t="n">
         <v>100</v>
       </c>
       <c r="W45" t="n">
-        <v>65.98</v>
+        <v>57</v>
       </c>
       <c r="X45" t="n">
-        <v>77.33</v>
+        <v>81.95999999999999</v>
       </c>
       <c r="Y45" t="inlineStr">
         <is>
@@ -62361,22 +62373,22 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>87.95999999999999</v>
+        <v>90.34999999999999</v>
       </c>
       <c r="T46" t="n">
-        <v>42.45</v>
+        <v>65.28</v>
       </c>
       <c r="U46" t="n">
-        <v>92.78</v>
+        <v>90.8</v>
       </c>
       <c r="V46" t="n">
         <v>66.67</v>
       </c>
       <c r="W46" t="n">
-        <v>63.84</v>
+        <v>57</v>
       </c>
       <c r="X46" t="n">
-        <v>69.43000000000001</v>
+        <v>74.41</v>
       </c>
       <c r="Y46" t="inlineStr">
         <is>
@@ -62455,30 +62467,30 @@
         <v>0</v>
       </c>
       <c r="S47" t="n">
-        <v>64.76000000000001</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="T47" t="n">
-        <v>76.16</v>
+        <v>87.61</v>
       </c>
       <c r="U47" t="n">
-        <v>78.16</v>
+        <v>78.54000000000001</v>
       </c>
       <c r="V47" t="n">
         <v>93.33</v>
       </c>
       <c r="W47" t="n">
-        <v>56.82</v>
+        <v>91</v>
       </c>
       <c r="X47" t="n">
-        <v>74.14</v>
+        <v>84.72</v>
       </c>
       <c r="Y47" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -62549,22 +62561,22 @@
         <v>0</v>
       </c>
       <c r="S48" t="n">
-        <v>69.01000000000001</v>
+        <v>77.5</v>
       </c>
       <c r="T48" t="n">
         <v>50</v>
       </c>
       <c r="U48" t="n">
-        <v>61.22</v>
+        <v>55.32</v>
       </c>
       <c r="V48" t="n">
         <v>0</v>
       </c>
       <c r="W48" t="n">
-        <v>68.69</v>
+        <v>91</v>
       </c>
       <c r="X48" t="n">
-        <v>49.24</v>
+        <v>53.82</v>
       </c>
       <c r="Y48" t="inlineStr">
         <is>
@@ -62643,26 +62655,26 @@
         <v>0</v>
       </c>
       <c r="S49" t="n">
-        <v>52.56</v>
+        <v>66.8</v>
       </c>
       <c r="T49" t="n">
-        <v>79.72</v>
+        <v>91.04000000000001</v>
       </c>
       <c r="U49" t="n">
-        <v>77.41</v>
+        <v>74.78</v>
       </c>
       <c r="V49" t="n">
         <v>100</v>
       </c>
       <c r="W49" t="n">
-        <v>59.99</v>
+        <v>88</v>
       </c>
       <c r="X49" t="n">
-        <v>73.68000000000001</v>
+        <v>83.88</v>
       </c>
       <c r="Y49" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z49" t="b">
@@ -62737,30 +62749,30 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>25.53</v>
+        <v>49</v>
       </c>
       <c r="T50" t="n">
-        <v>81.13</v>
+        <v>91.67</v>
       </c>
       <c r="U50" t="n">
-        <v>69</v>
+        <v>70.58</v>
       </c>
       <c r="V50" t="n">
         <v>33.33</v>
       </c>
       <c r="W50" t="n">
-        <v>71.19</v>
+        <v>82</v>
       </c>
       <c r="X50" t="n">
-        <v>54.36</v>
+        <v>64.72</v>
       </c>
       <c r="Y50" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -62831,26 +62843,26 @@
         <v>0</v>
       </c>
       <c r="S51" t="n">
-        <v>46.42</v>
+        <v>64.3</v>
       </c>
       <c r="T51" t="n">
-        <v>84.58</v>
+        <v>93.19</v>
       </c>
       <c r="U51" t="n">
-        <v>51.7</v>
+        <v>53.09</v>
       </c>
       <c r="V51" t="n">
         <v>83.33</v>
       </c>
       <c r="W51" t="n">
-        <v>51.16</v>
+        <v>94</v>
       </c>
       <c r="X51" t="n">
-        <v>64.84</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="Y51" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z51" t="b">
@@ -62925,22 +62937,22 @@
         <v>1</v>
       </c>
       <c r="S52" t="n">
-        <v>70.06999999999999</v>
+        <v>78.15000000000001</v>
       </c>
       <c r="T52" t="n">
-        <v>82.64</v>
+        <v>92.33</v>
       </c>
       <c r="U52" t="n">
-        <v>75.37</v>
+        <v>77.09</v>
       </c>
       <c r="V52" t="n">
         <v>100</v>
       </c>
       <c r="W52" t="n">
-        <v>58.15</v>
+        <v>61</v>
       </c>
       <c r="X52" t="n">
-        <v>78.20999999999999</v>
+        <v>83.33</v>
       </c>
       <c r="Y52" t="inlineStr">
         <is>
@@ -63019,22 +63031,22 @@
         <v>1</v>
       </c>
       <c r="S53" t="n">
-        <v>22.41</v>
+        <v>48.35</v>
       </c>
       <c r="T53" t="n">
-        <v>66.81999999999999</v>
+        <v>80.69</v>
       </c>
       <c r="U53" t="n">
-        <v>45.14</v>
+        <v>51.87</v>
       </c>
       <c r="V53" t="n">
         <v>100</v>
       </c>
       <c r="W53" t="n">
-        <v>67.3</v>
+        <v>58</v>
       </c>
       <c r="X53" t="n">
-        <v>59.17</v>
+        <v>68.73999999999999</v>
       </c>
       <c r="Y53" t="inlineStr">
         <is>
@@ -63113,26 +63125,26 @@
         <v>0</v>
       </c>
       <c r="S54" t="n">
-        <v>64.59999999999999</v>
+        <v>74.8</v>
       </c>
       <c r="T54" t="n">
-        <v>84.91</v>
+        <v>93.33</v>
       </c>
       <c r="U54" t="n">
-        <v>89.40000000000001</v>
+        <v>87.20999999999999</v>
       </c>
       <c r="V54" t="n">
         <v>100</v>
       </c>
       <c r="W54" t="n">
-        <v>26.75</v>
+        <v>91</v>
       </c>
       <c r="X54" t="n">
-        <v>74.8</v>
+        <v>88.76000000000001</v>
       </c>
       <c r="Y54" t="inlineStr">
         <is>
-          <t>Established</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="Z54" t="b">
@@ -63207,30 +63219,30 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>60.22</v>
+        <v>72.75</v>
       </c>
       <c r="T55" t="n">
-        <v>84.91</v>
+        <v>93.33</v>
       </c>
       <c r="U55" t="n">
-        <v>61.82</v>
+        <v>58.12</v>
       </c>
       <c r="V55" t="n">
         <v>0</v>
       </c>
       <c r="W55" t="n">
-        <v>44.21</v>
+        <v>94</v>
       </c>
       <c r="X55" t="n">
-        <v>52.19</v>
+        <v>64.34</v>
       </c>
       <c r="Y55" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Established</t>
         </is>
       </c>
       <c r="Z55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -63301,22 +63313,22 @@
         <v>1</v>
       </c>
       <c r="S56" t="n">
-        <v>42.08</v>
+        <v>58.5</v>
       </c>
       <c r="T56" t="n">
-        <v>52.36</v>
+        <v>65</v>
       </c>
       <c r="U56" t="n">
-        <v>71.77</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="V56" t="n">
         <v>100</v>
       </c>
       <c r="W56" t="n">
-        <v>50.49</v>
+        <v>49</v>
       </c>
       <c r="X56" t="n">
-        <v>61.95</v>
+        <v>68.94</v>
       </c>
       <c r="Y56" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Period-scoped chips, tier mismatch removed, absent suppliers in ranking + PT Gunung Raja Paksi synthetic data added
</commit_message>
<xml_diff>
--- a/data/raw/procurement_data.xlsx
+++ b/data/raw/procurement_data.xlsx
@@ -2233,7 +2233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U641"/>
+  <dimension ref="A1:U648"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58021,6 +58021,615 @@
       </c>
       <c r="U641" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>PO-2024-00901</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>S101</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>PT Gunung Raja Paksi</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Local Steel</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>Deformed rebar (BjTS 420)</t>
+        </is>
+      </c>
+      <c r="F642" t="inlineStr">
+        <is>
+          <t>tonne</t>
+        </is>
+      </c>
+      <c r="G642" t="n">
+        <v>120</v>
+      </c>
+      <c r="H642" t="n">
+        <v>850</v>
+      </c>
+      <c r="I642" t="n">
+        <v>102000</v>
+      </c>
+      <c r="J642" t="inlineStr">
+        <is>
+          <t>2024-03-04</t>
+        </is>
+      </c>
+      <c r="K642" t="inlineStr">
+        <is>
+          <t>2024-03-09</t>
+        </is>
+      </c>
+      <c r="L642" t="inlineStr">
+        <is>
+          <t>2024-03-19</t>
+        </is>
+      </c>
+      <c r="M642" t="inlineStr">
+        <is>
+          <t>2024-03-23</t>
+        </is>
+      </c>
+      <c r="N642" t="inlineStr">
+        <is>
+          <t>2024-04-10</t>
+        </is>
+      </c>
+      <c r="O642" t="n">
+        <v>5</v>
+      </c>
+      <c r="P642" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q642" t="n">
+        <v>4</v>
+      </c>
+      <c r="R642" t="n">
+        <v>18</v>
+      </c>
+      <c r="S642" t="n">
+        <v>37</v>
+      </c>
+      <c r="T642" t="b">
+        <v>1</v>
+      </c>
+      <c r="U642" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>PO-2024-00902</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>S101</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>PT Gunung Raja Paksi</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Local Steel</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>Structural H-beam steel</t>
+        </is>
+      </c>
+      <c r="F643" t="inlineStr">
+        <is>
+          <t>tonne</t>
+        </is>
+      </c>
+      <c r="G643" t="n">
+        <v>80</v>
+      </c>
+      <c r="H643" t="n">
+        <v>1100</v>
+      </c>
+      <c r="I643" t="n">
+        <v>88000</v>
+      </c>
+      <c r="J643" t="inlineStr">
+        <is>
+          <t>2024-08-12</t>
+        </is>
+      </c>
+      <c r="K643" t="inlineStr">
+        <is>
+          <t>2024-08-18</t>
+        </is>
+      </c>
+      <c r="L643" t="inlineStr">
+        <is>
+          <t>2024-08-30</t>
+        </is>
+      </c>
+      <c r="M643" t="inlineStr">
+        <is>
+          <t>2024-09-04</t>
+        </is>
+      </c>
+      <c r="N643" t="inlineStr">
+        <is>
+          <t>2024-09-24</t>
+        </is>
+      </c>
+      <c r="O643" t="n">
+        <v>6</v>
+      </c>
+      <c r="P643" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q643" t="n">
+        <v>5</v>
+      </c>
+      <c r="R643" t="n">
+        <v>20</v>
+      </c>
+      <c r="S643" t="n">
+        <v>43</v>
+      </c>
+      <c r="T643" t="b">
+        <v>1</v>
+      </c>
+      <c r="U643" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>PO-2025-00903</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>S101</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>PT Gunung Raja Paksi</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Local Steel</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>Hot-rolled steel plate</t>
+        </is>
+      </c>
+      <c r="F644" t="inlineStr">
+        <is>
+          <t>tonne</t>
+        </is>
+      </c>
+      <c r="G644" t="n">
+        <v>150</v>
+      </c>
+      <c r="H644" t="n">
+        <v>950</v>
+      </c>
+      <c r="I644" t="n">
+        <v>142500</v>
+      </c>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>2025-02-10</t>
+        </is>
+      </c>
+      <c r="K644" t="inlineStr">
+        <is>
+          <t>2025-02-17</t>
+        </is>
+      </c>
+      <c r="L644" t="inlineStr">
+        <is>
+          <t>2025-03-09</t>
+        </is>
+      </c>
+      <c r="M644" t="inlineStr">
+        <is>
+          <t>2025-03-15</t>
+        </is>
+      </c>
+      <c r="N644" t="inlineStr">
+        <is>
+          <t>2025-03-30</t>
+        </is>
+      </c>
+      <c r="O644" t="n">
+        <v>7</v>
+      </c>
+      <c r="P644" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q644" t="n">
+        <v>6</v>
+      </c>
+      <c r="R644" t="n">
+        <v>15</v>
+      </c>
+      <c r="S644" t="n">
+        <v>48</v>
+      </c>
+      <c r="T644" t="b">
+        <v>0</v>
+      </c>
+      <c r="U644" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>PO-2025-00904</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>S101</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>PT Gunung Raja Paksi</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Local Steel</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Cold-rolled steel coil</t>
+        </is>
+      </c>
+      <c r="F645" t="inlineStr">
+        <is>
+          <t>tonne</t>
+        </is>
+      </c>
+      <c r="G645" t="n">
+        <v>200</v>
+      </c>
+      <c r="H645" t="n">
+        <v>1050</v>
+      </c>
+      <c r="I645" t="n">
+        <v>210000</v>
+      </c>
+      <c r="J645" t="inlineStr">
+        <is>
+          <t>2025-06-03</t>
+        </is>
+      </c>
+      <c r="K645" t="inlineStr">
+        <is>
+          <t>2025-06-07</t>
+        </is>
+      </c>
+      <c r="L645" t="inlineStr">
+        <is>
+          <t>2025-06-20</t>
+        </is>
+      </c>
+      <c r="M645" t="inlineStr">
+        <is>
+          <t>2025-06-23</t>
+        </is>
+      </c>
+      <c r="N645" t="inlineStr">
+        <is>
+          <t>2025-07-15</t>
+        </is>
+      </c>
+      <c r="O645" t="n">
+        <v>4</v>
+      </c>
+      <c r="P645" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q645" t="n">
+        <v>3</v>
+      </c>
+      <c r="R645" t="n">
+        <v>22</v>
+      </c>
+      <c r="S645" t="n">
+        <v>42</v>
+      </c>
+      <c r="T645" t="b">
+        <v>1</v>
+      </c>
+      <c r="U645" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>PO-2025-00905</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>S101</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>PT Gunung Raja Paksi</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Local Steel</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>Steel angle bar</t>
+        </is>
+      </c>
+      <c r="F646" t="inlineStr">
+        <is>
+          <t>tonne</t>
+        </is>
+      </c>
+      <c r="G646" t="n">
+        <v>90</v>
+      </c>
+      <c r="H646" t="n">
+        <v>900</v>
+      </c>
+      <c r="I646" t="n">
+        <v>81000</v>
+      </c>
+      <c r="J646" t="inlineStr">
+        <is>
+          <t>2025-10-06</t>
+        </is>
+      </c>
+      <c r="K646" t="inlineStr">
+        <is>
+          <t>2025-10-14</t>
+        </is>
+      </c>
+      <c r="L646" t="inlineStr">
+        <is>
+          <t>2025-10-28</t>
+        </is>
+      </c>
+      <c r="M646" t="inlineStr">
+        <is>
+          <t>2025-11-02</t>
+        </is>
+      </c>
+      <c r="N646" t="inlineStr">
+        <is>
+          <t>2025-11-21</t>
+        </is>
+      </c>
+      <c r="O646" t="n">
+        <v>8</v>
+      </c>
+      <c r="P646" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q646" t="n">
+        <v>5</v>
+      </c>
+      <c r="R646" t="n">
+        <v>19</v>
+      </c>
+      <c r="S646" t="n">
+        <v>46</v>
+      </c>
+      <c r="T646" t="b">
+        <v>1</v>
+      </c>
+      <c r="U646" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>PO-2026-00906</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>S101</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>PT Gunung Raja Paksi</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Local Steel</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Galvanized steel sheet</t>
+        </is>
+      </c>
+      <c r="F647" t="inlineStr">
+        <is>
+          <t>tonne</t>
+        </is>
+      </c>
+      <c r="G647" t="n">
+        <v>110</v>
+      </c>
+      <c r="H647" t="n">
+        <v>1200</v>
+      </c>
+      <c r="I647" t="n">
+        <v>132000</v>
+      </c>
+      <c r="J647" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="K647" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="L647" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="M647" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="N647" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="O647" t="n">
+        <v>5</v>
+      </c>
+      <c r="P647" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q647" t="n">
+        <v>4</v>
+      </c>
+      <c r="R647" t="n">
+        <v>16</v>
+      </c>
+      <c r="S647" t="n">
+        <v>34</v>
+      </c>
+      <c r="T647" t="b">
+        <v>1</v>
+      </c>
+      <c r="U647" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>PO-2026-00907</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>S101</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>PT Gunung Raja Paksi</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Local Steel</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>Hot-rolled steel plate</t>
+        </is>
+      </c>
+      <c r="F648" t="inlineStr">
+        <is>
+          <t>tonne</t>
+        </is>
+      </c>
+      <c r="G648" t="n">
+        <v>170</v>
+      </c>
+      <c r="H648" t="n">
+        <v>800</v>
+      </c>
+      <c r="I648" t="n">
+        <v>136000</v>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="K648" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="L648" t="inlineStr">
+        <is>
+          <t>2026-04-06</t>
+        </is>
+      </c>
+      <c r="M648" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="N648" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="O648" t="n">
+        <v>6</v>
+      </c>
+      <c r="P648" t="n">
+        <v>22</v>
+      </c>
+      <c r="Q648" t="n">
+        <v>7</v>
+      </c>
+      <c r="R648" t="n">
+        <v>21</v>
+      </c>
+      <c r="S648" t="n">
+        <v>56</v>
+      </c>
+      <c r="T648" t="b">
+        <v>0</v>
+      </c>
+      <c r="U648" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -58034,7 +58643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z56"/>
+  <dimension ref="A1:X56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58158,16 +58767,6 @@
           <t>composite_score</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>calculated_tier</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>tier_mismatch</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -58254,14 +58853,6 @@
       <c r="X2" t="n">
         <v>90.17</v>
       </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z2" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -58348,14 +58939,6 @@
       <c r="X3" t="n">
         <v>89.05</v>
       </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z3" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -58442,14 +59025,6 @@
       <c r="X4" t="n">
         <v>86.51000000000001</v>
       </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z4" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -58536,14 +59111,6 @@
       <c r="X5" t="n">
         <v>80.84999999999999</v>
       </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z5" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -58630,14 +59197,6 @@
       <c r="X6" t="n">
         <v>74</v>
       </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z6" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -58724,14 +59283,6 @@
       <c r="X7" t="n">
         <v>78.63</v>
       </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z7" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -58818,14 +59369,6 @@
       <c r="X8" t="n">
         <v>79.09999999999999</v>
       </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z8" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -58912,14 +59455,6 @@
       <c r="X9" t="n">
         <v>76.61</v>
       </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z9" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -59006,14 +59541,6 @@
       <c r="X10" t="n">
         <v>82.61</v>
       </c>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z10" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -59100,14 +59627,6 @@
       <c r="X11" t="n">
         <v>79.69</v>
       </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z11" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -59194,14 +59713,6 @@
       <c r="X12" t="n">
         <v>83.78</v>
       </c>
-      <c r="Y12" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z12" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -59288,14 +59799,6 @@
       <c r="X13" t="n">
         <v>67.79000000000001</v>
       </c>
-      <c r="Y13" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z13" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -59382,14 +59885,6 @@
       <c r="X14" t="n">
         <v>76.91</v>
       </c>
-      <c r="Y14" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z14" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -59476,14 +59971,6 @@
       <c r="X15" t="n">
         <v>81.05</v>
       </c>
-      <c r="Y15" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z15" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -59570,14 +60057,6 @@
       <c r="X16" t="n">
         <v>83.31999999999999</v>
       </c>
-      <c r="Y16" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z16" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -59664,14 +60143,6 @@
       <c r="X17" t="n">
         <v>72.29000000000001</v>
       </c>
-      <c r="Y17" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z17" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -59758,14 +60229,6 @@
       <c r="X18" t="n">
         <v>85.56999999999999</v>
       </c>
-      <c r="Y18" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z18" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -59852,14 +60315,6 @@
       <c r="X19" t="n">
         <v>72.81999999999999</v>
       </c>
-      <c r="Y19" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z19" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -59946,14 +60401,6 @@
       <c r="X20" t="n">
         <v>76.63</v>
       </c>
-      <c r="Y20" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z20" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -60040,14 +60487,6 @@
       <c r="X21" t="n">
         <v>73.28</v>
       </c>
-      <c r="Y21" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z21" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -60134,14 +60573,6 @@
       <c r="X22" t="n">
         <v>75.31999999999999</v>
       </c>
-      <c r="Y22" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z22" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -60228,14 +60659,6 @@
       <c r="X23" t="n">
         <v>66.88</v>
       </c>
-      <c r="Y23" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z23" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -60322,14 +60745,6 @@
       <c r="X24" t="n">
         <v>87.90000000000001</v>
       </c>
-      <c r="Y24" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z24" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -60416,14 +60831,6 @@
       <c r="X25" t="n">
         <v>86.64</v>
       </c>
-      <c r="Y25" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z25" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -60510,14 +60917,6 @@
       <c r="X26" t="n">
         <v>82.87</v>
       </c>
-      <c r="Y26" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z26" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -60604,14 +61003,6 @@
       <c r="X27" t="n">
         <v>83.38</v>
       </c>
-      <c r="Y27" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z27" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -60698,14 +61089,6 @@
       <c r="X28" t="n">
         <v>77.84</v>
       </c>
-      <c r="Y28" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z28" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -60792,14 +61175,6 @@
       <c r="X29" t="n">
         <v>72.97</v>
       </c>
-      <c r="Y29" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z29" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -60886,14 +61261,6 @@
       <c r="X30" t="n">
         <v>71.86</v>
       </c>
-      <c r="Y30" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z30" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -60980,14 +61347,6 @@
       <c r="X31" t="n">
         <v>80.03</v>
       </c>
-      <c r="Y31" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z31" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -61074,14 +61433,6 @@
       <c r="X32" t="n">
         <v>80.44</v>
       </c>
-      <c r="Y32" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z32" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -61168,14 +61519,6 @@
       <c r="X33" t="n">
         <v>66.64</v>
       </c>
-      <c r="Y33" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z33" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -61262,14 +61605,6 @@
       <c r="X34" t="n">
         <v>63.3</v>
       </c>
-      <c r="Y34" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z34" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -61356,14 +61691,6 @@
       <c r="X35" t="n">
         <v>68.23</v>
       </c>
-      <c r="Y35" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z35" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -61450,14 +61777,6 @@
       <c r="X36" t="n">
         <v>68.13</v>
       </c>
-      <c r="Y36" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z36" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -61544,14 +61863,6 @@
       <c r="X37" t="n">
         <v>74.83</v>
       </c>
-      <c r="Y37" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z37" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -61638,14 +61949,6 @@
       <c r="X38" t="n">
         <v>52.66</v>
       </c>
-      <c r="Y38" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="Z38" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -61732,14 +62035,6 @@
       <c r="X39" t="n">
         <v>78.45</v>
       </c>
-      <c r="Y39" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z39" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -61826,14 +62121,6 @@
       <c r="X40" t="n">
         <v>69.63</v>
       </c>
-      <c r="Y40" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z40" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -61920,14 +62207,6 @@
       <c r="X41" t="n">
         <v>73.34</v>
       </c>
-      <c r="Y41" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z41" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -62014,14 +62293,6 @@
       <c r="X42" t="n">
         <v>71.75</v>
       </c>
-      <c r="Y42" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z42" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -62108,14 +62379,6 @@
       <c r="X43" t="n">
         <v>75.62</v>
       </c>
-      <c r="Y43" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z43" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -62202,14 +62465,6 @@
       <c r="X44" t="n">
         <v>80.75</v>
       </c>
-      <c r="Y44" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z44" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -62296,14 +62551,6 @@
       <c r="X45" t="n">
         <v>81.95999999999999</v>
       </c>
-      <c r="Y45" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z45" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -62390,14 +62637,6 @@
       <c r="X46" t="n">
         <v>74.41</v>
       </c>
-      <c r="Y46" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z46" t="b">
-        <v>0</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -62484,14 +62723,6 @@
       <c r="X47" t="n">
         <v>84.72</v>
       </c>
-      <c r="Y47" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z47" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -62525,66 +62756,58 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>0</v>
+        <v>891500</v>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
+        <v>127357.14</v>
       </c>
       <c r="J48" t="n">
-        <v>0</v>
+        <v>14.29</v>
       </c>
       <c r="K48" t="n">
-        <v>0</v>
+        <v>43.71</v>
       </c>
       <c r="L48" t="n">
-        <v>0</v>
+        <v>71.43000000000001</v>
       </c>
       <c r="M48" t="n">
-        <v>0</v>
+        <v>85.70999999999999</v>
       </c>
       <c r="N48" t="n">
-        <v>1.5</v>
+        <v>3.8</v>
       </c>
       <c r="O48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P48" t="n">
-        <v>86.20999999999999</v>
+        <v>68</v>
       </c>
       <c r="Q48" t="n">
-        <v>10.58</v>
+        <v>4</v>
       </c>
       <c r="R48" t="n">
         <v>0</v>
       </c>
       <c r="S48" t="n">
-        <v>77.5</v>
+        <v>71</v>
       </c>
       <c r="T48" t="n">
-        <v>50</v>
+        <v>73.81</v>
       </c>
       <c r="U48" t="n">
-        <v>55.32</v>
+        <v>69.70999999999999</v>
       </c>
       <c r="V48" t="n">
-        <v>0</v>
+        <v>85.70999999999999</v>
       </c>
       <c r="W48" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="X48" t="n">
-        <v>53.82</v>
-      </c>
-      <c r="Y48" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="Z48" t="b">
-        <v>0</v>
+        <v>77.90000000000001</v>
       </c>
     </row>
     <row r="49">
@@ -62672,14 +62895,6 @@
       <c r="X49" t="n">
         <v>83.88</v>
       </c>
-      <c r="Y49" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z49" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -62766,14 +62981,6 @@
       <c r="X50" t="n">
         <v>64.72</v>
       </c>
-      <c r="Y50" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z50" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -62860,14 +63067,6 @@
       <c r="X51" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="Y51" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z51" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -62954,14 +63153,6 @@
       <c r="X52" t="n">
         <v>83.33</v>
       </c>
-      <c r="Y52" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z52" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -63048,14 +63239,6 @@
       <c r="X53" t="n">
         <v>68.73999999999999</v>
       </c>
-      <c r="Y53" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z53" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -63142,14 +63325,6 @@
       <c r="X54" t="n">
         <v>88.76000000000001</v>
       </c>
-      <c r="Y54" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
-      <c r="Z54" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -63236,14 +63411,6 @@
       <c r="X55" t="n">
         <v>64.34</v>
       </c>
-      <c r="Y55" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z55" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -63329,14 +63496,6 @@
       </c>
       <c r="X56" t="n">
         <v>68.94</v>
-      </c>
-      <c r="Y56" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
-      <c r="Z56" t="b">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>